<commit_message>
feat(data): CĐ2 tables -> Excel (15 sheets); improve markdown-table extractor
- dist/figure_data/cd2_tables.xlsx — README + 15 sheets: all CĐ2 content tables
  (Bảng 2.1–2.13: theory layers, I–P functional forms, variable mapping, H1–H6
  hypothesis system, CDCM predictions, 8 models M0–M7, ICRV pool structure, TCI/DAI
  measurement, 50-economy ICRV classification, robustness plan) + the abbreviations
  list + the predicted-turning-point-by-ICRV table. Verbatim parse; the per-ICRV
  TP table carries the canonical P7 values (M5 43.6% / N=79,080; M2 N=81,022).
- scripts/extract_markdown_tables.py — now recognises non-bold 'Bảng X.N' captions
  and '## Headings', and falls back to header-cell naming when no caption exists.
  Refreshed the Chương 3 workbook with the improved naming.
</commit_message>
<xml_diff>
--- a/dist/figure_data/chuong3_phuong_phap_tables.xlsx
+++ b/dist/figure_data/chuong3_phuong_phap_tables.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C35_Ký_hiệu_biến_tiếng_Việt" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C36_Phân_tích_độ_vững_kiểm_t" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C37_Bảng_định_nghĩa_biến_Ngh" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C38_C38" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C38_36_Tóm_tắt_phương_pháp_K" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -549,10 +549,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C38_C38</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
+          <t>C38_36_Tóm_tắt_phương_pháp_K</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>3.6 Tóm tắt phương pháp: Kế thừa và đóng góp mới</t>
+        </is>
+      </c>
       <c r="C9" t="n">
         <v>11</v>
       </c>

</xml_diff>